<commit_message>
chore: #117을 #30으로 통합 반영 — Excel/JSON 최신화
- #117 「가공도 단면 위주 출력·은선 정책」을 #30 중복으로 종료.
  본문에 단면 정책 내용이 없고 형상 누락 증상만 있었으며, 사용자 확인 결과
  가공도 한정이 아니라 모든 2D Drawing에서 나오는 문제라 분리 근거가 무너짐
- #30에 `도면: 가공도` 추가, 증상을 "2D 변환을 거치는 모든 출력"으로 정정,
  도면 종류별 검증(제작·조립·설치·가공)을 완료 조건 체크로 흡수

집계: 열린 이슈 57, 필수 9건 (개발사 7 / 내부 3, #42는 양쪽)
사내 Daily review 9줄과 1:1 대응 완성

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/개발 현황.xlsx
+++ b/개발 현황.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이슈 목록" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'이슈 목록'!$A$1:$P$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'이슈 목록'!$A$1:$P$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>생성 시각 2026-07-30 14:01 · 원천은 GitHub 이슈이며 이 파일은 읽기 전용 생성물입니다. 손으로 고치지 마십시오.</t>
+          <t>생성 시각 2026-07-30 14:13 · 원천은 GitHub 이슈이며 이 파일은 읽기 전용 생성물입니다. 손으로 고치지 마십시오.</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -573,7 +573,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>68.9%</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -809,12 +809,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>가공도</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -953,11 +953,11 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>가공도 단면 위주 출력·은선 정책</t>
+          <t>No Paint 표시방법 — 도면 표기 방식 확정</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>가공도</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -982,27 +982,27 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/uuuuj/a2z/issues/117</t>
+          <t>https://github.com/uuuuj/a2z/issues/197</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>197</v>
+        <v>111</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>No Paint 표시방법 — 도면 표기 방식 확정</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>API 개발</t>
+          <t>PNOD 표시 — 값이 담긴 att(UDA) 키·노드 레벨 확인</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>내부 해결</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>API 대기</t>
+          <t>분석 필요</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1017,17 +1017,17 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/uuuuj/a2z/issues/197</t>
+          <t>https://github.com/uuuuj/a2z/issues/111</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>111</v>
+        <v>198</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>PNOD 표시 — 값이 담긴 att(UDA) 키·노드 레벨 확인</t>
+          <t>개발에 필요한 att(UDA) 속성 정리 — 모델 변환 쪽에 일괄 요청</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -1051,41 +1051,6 @@
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>https://github.com/uuuuj/a2z/issues/111</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>198</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>개발에 필요한 att(UDA) 속성 정리 — 모델 변환 쪽에 일괄 요청</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>내부 해결</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>분석 필요</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>공통</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>https://github.com/uuuuj/a2z/issues/198</t>
         </is>
@@ -1102,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P197"/>
+  <dimension ref="A1:P199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2561,7 +2526,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>가공도</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -2586,7 +2551,7 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Excel No.14</t>
+          <t>Excel No.14, 64</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2602,7 +2567,7 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="N28" s="5" t="n">
@@ -4730,7 +4695,7 @@
         </is>
       </c>
       <c r="N68" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
@@ -7814,7 +7779,7 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>API 대기</t>
+          <t>미채택</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
@@ -7827,16 +7792,8 @@
           <t>O</t>
         </is>
       </c>
-      <c r="F115" s="5" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>API 개발</t>
-        </is>
-      </c>
+      <c r="F115" s="5" t="inlineStr"/>
+      <c r="G115" s="5" t="inlineStr"/>
       <c r="H115" s="5" t="inlineStr">
         <is>
           <t>뷰</t>
@@ -7852,7 +7809,11 @@
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="K115" s="5" t="inlineStr"/>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="L115" s="5" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -7860,15 +7821,15 @@
       </c>
       <c r="M115" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="N115" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O115" s="5" t="inlineStr">
         <is>
-          <t>생산 필수, backfill</t>
+          <t>duplicate, 생산 필수, backfill</t>
         </is>
       </c>
       <c r="P115" s="5" t="inlineStr">
@@ -12285,8 +12246,116 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="B198" s="6" t="inlineStr">
+        <is>
+          <t>ClickOnce 게시에 네이티브 DLL 5종 누락 — 설치는 되나 실행 즉시 종료</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>개발 대기</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr"/>
+      <c r="E198" s="11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F198" s="5" t="inlineStr"/>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>내부 해결</t>
+        </is>
+      </c>
+      <c r="H198" s="5" t="inlineStr"/>
+      <c r="I198" s="5" t="inlineStr"/>
+      <c r="J198" s="5" t="inlineStr"/>
+      <c r="K198" s="5" t="inlineStr"/>
+      <c r="L198" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="M198" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="N198" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O198" s="5" t="inlineStr">
+        <is>
+          <t>생산 필수</t>
+        </is>
+      </c>
+      <c r="P198" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/uuuuj/a2z/issues/200</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="n">
+        <v>201</v>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>ClickOnce 설치 시 도면·로그 출력 위치 — 담당자가 결과물을 찾을 수 없음</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>분석 필요</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr"/>
+      <c r="E199" s="11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F199" s="5" t="inlineStr"/>
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>내부 해결</t>
+        </is>
+      </c>
+      <c r="H199" s="5" t="inlineStr"/>
+      <c r="I199" s="5" t="inlineStr"/>
+      <c r="J199" s="5" t="inlineStr"/>
+      <c r="K199" s="5" t="inlineStr"/>
+      <c r="L199" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="M199" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="N199" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O199" s="5" t="inlineStr">
+        <is>
+          <t>생산 필수</t>
+        </is>
+      </c>
+      <c r="P199" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/uuuuj/a2z/issues/201</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P197"/>
+  <autoFilter ref="A1:P199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>